<commit_message>
Add 10 portfolio management articles + index
</commit_message>
<xml_diff>
--- a/Cluenex Content.xlsx
+++ b/Cluenex Content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Claude\Projects\Cluenex Content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A60BD60B-0852-4EF6-84A8-F3D0D0710FAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCFD201-F705-491B-8C84-962BC5F1E1E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{98ACFBED-9EB7-4642-8712-CDA9C50EE277}"/>
   </bookViews>
@@ -2033,7 +2033,7 @@
       <c r="U53" s="2"/>
     </row>
     <row r="54" spans="2:21">
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C54" s="3"/>
@@ -2048,7 +2048,7 @@
       <c r="U54" s="2"/>
     </row>
     <row r="55" spans="2:21">
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>40</v>
       </c>
       <c r="C55" s="3"/>
@@ -2065,7 +2065,7 @@
       <c r="U55" s="2"/>
     </row>
     <row r="56" spans="2:21">
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="4" t="s">
         <v>41</v>
       </c>
       <c r="C56" s="3"/>
@@ -2082,7 +2082,7 @@
       <c r="U56" s="2"/>
     </row>
     <row r="57" spans="2:21">
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="4" t="s">
         <v>42</v>
       </c>
       <c r="C57" s="3"/>
@@ -2099,7 +2099,7 @@
       <c r="U57" s="2"/>
     </row>
     <row r="58" spans="2:21">
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C58" s="3"/>
@@ -2116,7 +2116,7 @@
       <c r="U58" s="2"/>
     </row>
     <row r="59" spans="2:21">
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="4" t="s">
         <v>44</v>
       </c>
       <c r="C59" s="3"/>
@@ -2133,7 +2133,7 @@
       <c r="U59" s="2"/>
     </row>
     <row r="60" spans="2:21">
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>45</v>
       </c>
       <c r="C60" s="3"/>
@@ -2150,7 +2150,7 @@
       <c r="U60" s="2"/>
     </row>
     <row r="61" spans="2:21">
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="4" t="s">
         <v>46</v>
       </c>
       <c r="C61" s="3"/>
@@ -2166,7 +2166,7 @@
       </c>
     </row>
     <row r="62" spans="2:21">
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="4" t="s">
         <v>47</v>
       </c>
       <c r="C62" s="3"/>
@@ -2182,7 +2182,7 @@
       </c>
     </row>
     <row r="63" spans="2:21">
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="4" t="s">
         <v>48</v>
       </c>
       <c r="C63" s="3"/>
@@ -2198,7 +2198,7 @@
       </c>
     </row>
     <row r="64" spans="2:21">
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C64" s="3"/>
@@ -2214,7 +2214,7 @@
       </c>
     </row>
     <row r="65" spans="2:15">
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="4" t="s">
         <v>50</v>
       </c>
       <c r="C65" s="3"/>
@@ -2227,7 +2227,7 @@
       <c r="J65" s="3"/>
     </row>
     <row r="66" spans="2:15">
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C66" s="3"/>
@@ -2243,7 +2243,7 @@
       </c>
     </row>
     <row r="67" spans="2:15">
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C67" s="3"/>
@@ -2257,7 +2257,7 @@
       <c r="O67" s="2"/>
     </row>
     <row r="68" spans="2:15">
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="4" t="s">
         <v>53</v>
       </c>
       <c r="C68" s="3"/>
@@ -2837,12 +2837,12 @@
       </c>
     </row>
     <row r="119" spans="2:15">
-      <c r="B119" s="2" t="s">
+      <c r="B119" s="4" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="120" spans="2:15">
-      <c r="B120" s="2" t="s">
+      <c r="B120" s="4" t="s">
         <v>89</v>
       </c>
       <c r="O120" s="3" t="s">
@@ -2850,13 +2850,13 @@
       </c>
     </row>
     <row r="121" spans="2:15">
-      <c r="B121" s="2" t="s">
+      <c r="B121" s="4" t="s">
         <v>90</v>
       </c>
       <c r="O121" s="2"/>
     </row>
     <row r="122" spans="2:15">
-      <c r="B122" s="2" t="s">
+      <c r="B122" s="4" t="s">
         <v>91</v>
       </c>
       <c r="O122" s="2" t="s">
@@ -2864,7 +2864,7 @@
       </c>
     </row>
     <row r="123" spans="2:15">
-      <c r="B123" s="2" t="s">
+      <c r="B123" s="4" t="s">
         <v>92</v>
       </c>
       <c r="O123" s="2" t="s">
@@ -2872,7 +2872,7 @@
       </c>
     </row>
     <row r="124" spans="2:15">
-      <c r="B124" s="2" t="s">
+      <c r="B124" s="4" t="s">
         <v>93</v>
       </c>
       <c r="O124" s="2" t="s">
@@ -2880,7 +2880,7 @@
       </c>
     </row>
     <row r="125" spans="2:15">
-      <c r="B125" s="2" t="s">
+      <c r="B125" s="4" t="s">
         <v>94</v>
       </c>
       <c r="O125" s="2" t="s">
@@ -2888,7 +2888,7 @@
       </c>
     </row>
     <row r="126" spans="2:15">
-      <c r="B126" s="2" t="s">
+      <c r="B126" s="4" t="s">
         <v>95</v>
       </c>
       <c r="O126" s="2" t="s">
@@ -2896,12 +2896,12 @@
       </c>
     </row>
     <row r="127" spans="2:15">
-      <c r="B127" s="2" t="s">
+      <c r="B127" s="4" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="128" spans="2:15">
-      <c r="B128" s="2" t="s">
+      <c r="B128" s="4" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>